<commit_message>
Fatto alcuni cambiamenti, palesemente il problema è nel calcolo del ritardo con aggiorna_schedulazione
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
+++ b/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -474,10 +474,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>253974</v>
+        <v>254187</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>45980.58333333334</v>
+        <v>45975.58333333334</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -485,34 +485,12 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>254187</v>
+        <v>254967</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>45975.58333333334</v>
+        <v>45981.58333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>254547</v>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>45980.58333333334</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>254967</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>45981.58333333334</v>
-      </c>
-      <c r="C5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
PROVA - cambiamenti apportati al bilanciamento della funzione obiettivo per il GRASP
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
+++ b/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -474,10 +474,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>254967</v>
+        <v>254671</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>45981.58333333334</v>
+        <v>45979.58333333334</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -485,21 +485,23 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>254671</v>
+        <v>254427</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
+        <v>45978.58333333334</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>253974</v>
+        <v>254173</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>45980.58333333334</v>
+        <v>45976.58333333334</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -507,127 +509,15 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>254101</v>
+        <v>254428</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>254100</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>254354</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>254252</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>254427</v>
-      </c>
-      <c r="B9" s="1" t="n">
         <v>45978.58333333334</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>253906</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>254428</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>45978.58333333334</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>254339</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>254547</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>45980.58333333334</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>254419</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>254173</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>45976.58333333334</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NB: rivedere calcolo_delta; non torna come è calcolato delta
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
+++ b/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
@@ -489,7 +489,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>254427</v>
+        <v>254428</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>45978.58333333334</v>
@@ -497,7 +497,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>254428</v>
+        <v>254427</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>45978.58333333334</v>

</xml_diff>

<commit_message>
NUOVA - calcolo rivisto
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
+++ b/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
@@ -447,9 +447,190 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>release_date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tassativita</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>254671</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>45979.58333333334</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>254967</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>45981.58333333334</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>253974</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>45980.58333333334</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>254100</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>45979.58333333334</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>254101</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>45979.58333333334</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>254354</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>45979.58333333334</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>254252</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>45979.58333333334</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>254428</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>45978.58333333334</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>254339</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>45979.58333333334</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>254173</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>45976.58333333334</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>254547</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>45980.58333333334</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>253906</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>45979.58333333334</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>254419</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>45979.58333333334</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>254427</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>45978.58333333334</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -489,7 +670,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>254428</v>
+        <v>254427</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>45978.58333333334</v>
@@ -497,7 +678,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>254427</v>
+        <v>254428</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>45978.58333333334</v>

</xml_diff>

<commit_message>
NUOVA - correzioni al GRASP
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
+++ b/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
@@ -418,25 +418,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>253940</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -447,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -474,10 +458,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>254671</v>
+        <v>253408</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>45979.58333333334</v>
+        <v>46000.58333333334</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -485,10 +469,10 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>254967</v>
+        <v>253902</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>45981.58333333334</v>
+        <v>46001.58333333334</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -496,138 +480,13 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>253974</v>
+        <v>255293</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>45980.58333333334</v>
+        <v>45991.58333333334</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>254100</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>254101</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>254354</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>254252</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>254428</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>45978.58333333334</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>254339</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>254173</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>45976.58333333334</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>254547</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>45980.58333333334</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>253906</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>254419</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>254427</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>45978.58333333334</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -641,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -662,26 +521,66 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>254237</v>
+        <v>254585</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>45975.58333333334</v>
+        <v>45994.58333333334</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>254427</v>
+        <v>254582</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>45978.58333333334</v>
+        <v>45994.58333333334</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>254428</v>
+        <v>254898</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>45978.58333333334</v>
+        <v>45994.58333333334</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>254911</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>45994.58333333334</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>254551</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>45994.58333333334</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>254978</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>45994.58333333334</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>254708</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>45995.58333333334</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>255220</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>45994.58333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NUOVO - .exe funzionante
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
+++ b/PS-VRP/Dati_output/Problemi_schedulazione_commesse.xlsx
@@ -447,190 +447,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>release_date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>tassativita</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>254967</v>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>45981.58333333334</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>254671</v>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>254354</v>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>253974</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>45980.58333333334</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>254101</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>254100</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>254252</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>254547</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>45980.58333333334</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>254419</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>254428</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>45978.58333333334</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>254427</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>45978.58333333334</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>253906</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>254173</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>45976.58333333334</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>254339</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>45979.58333333334</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>